<commit_message>
Corrige a paleta do war-room.html para bater com a referência visual
Fundo quase-preto (#07070f) com glows radiais roxo/magenta/azul e textura de
pontos; brand mark, tab ativa, botões primários e toggles agora usam um
gradiente azul→violeta→magenta (novas variáveis --violet/--magenta/--blue/
--gradient). As cores categóricas dos gráficos (validadas p/ daltonismo pela
skill dataviz) não foram alteradas — só a identidade visual/chrome.
</commit_message>
<xml_diff>
--- a/war-room-concorrencia/contexto-e-apoio/arquivos-finais/war-room.xlsx
+++ b/war-room-concorrencia/contexto-e-apoio/arquivos-finais/war-room.xlsx
@@ -2411,7 +2411,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Gerado em 2026-08-01 09:56 UTC | cadência sugerida: 6h</t>
+          <t>Gerado em 2026-08-01 10:11 UTC | cadência sugerida: 6h</t>
         </is>
       </c>
     </row>
@@ -3027,7 +3027,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-01 09:56 UTC</t>
+          <t>2026-08-01 10:11 UTC</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-01 09:56 UTC</t>
+          <t>2026-08-01 10:11 UTC</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-01 09:56 UTC</t>
+          <t>2026-08-01 10:11 UTC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-01 09:56 UTC</t>
+          <t>2026-08-01 10:11 UTC</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-01 09:56 UTC</t>
+          <t>2026-08-01 10:11 UTC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-01 09:56 UTC</t>
+          <t>2026-08-01 10:11 UTC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3968,185 +3968,185 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Faciderm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Black Skull</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="E2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F2" t="n">
+        <v>365</v>
+      </c>
+      <c r="G2" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Faciderm</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Growth Supplements</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Faciderm</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>NÓS</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>149.9</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>210</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H4" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>desconhecido</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Amaze</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Black Skull</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
         <v>84.90000000000001</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E5" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F5" t="n">
         <v>95</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G5" t="n">
         <v>4.3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Amaze</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>NÓS</t>
         </is>
       </c>
-      <c r="C3" s="11" t="n">
+      <c r="C6" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="11" t="n">
+      <c r="D6" s="11" t="n">
         <v>99.90000000000001</v>
       </c>
-      <c r="E3" s="11" t="n">
+      <c r="E6" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="11" t="n">
+      <c r="F6" s="11" t="n">
         <v>340</v>
       </c>
-      <c r="G3" s="11" t="n">
+      <c r="G6" s="11" t="n">
         <v>4.8</v>
       </c>
-      <c r="H3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="H6" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>desconhecido</t>
         </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Linha Joie Fit</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Black Skull</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>129.9</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>910</v>
-      </c>
-      <c r="G4" t="n">
-        <v>4.8</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Linha Joie Fit</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>NÓS</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>129.9</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="11" t="n">
-        <v>480</v>
-      </c>
-      <c r="G5" s="11" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H5" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>desconhecido</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Faciderm</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Black Skull</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>71.90000000000001</v>
-      </c>
-      <c r="E6" t="n">
-        <v>20</v>
-      </c>
-      <c r="F6" t="n">
-        <v>365</v>
-      </c>
-      <c r="G6" t="n">
-        <v>4.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Faciderm</t>
+          <t>Linha Joie Fit</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Growth Supplements</t>
+          <t>Black Skull</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>68.90000000000001</v>
+        <v>129.9</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>12</v>
+        <v>910</v>
       </c>
       <c r="G7" t="n">
-        <v>4.4</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Faciderm</t>
+          <t>Linha Joie Fit</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -4155,22 +4155,22 @@
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>149.9</v>
+        <v>129.9</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>210</v>
+        <v>480</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="H8" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
@@ -4497,105 +4497,105 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Faciderm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Black Skull</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="E2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F2" t="n">
+        <v>210</v>
+      </c>
+      <c r="G2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Faciderm</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>NÓS</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>149.9</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Amaze</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>NÓS</t>
         </is>
       </c>
-      <c r="C2" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="11" t="n">
+      <c r="C4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="11" t="n">
         <v>99.90000000000001</v>
       </c>
-      <c r="E2" s="11" t="n">
+      <c r="E4" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F2" s="11" t="n">
+      <c r="F4" s="11" t="n">
         <v>150</v>
       </c>
-      <c r="G2" s="11" t="n">
+      <c r="G4" s="11" t="n">
         <v>4.8</v>
       </c>
-      <c r="H2" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="11" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Amaze</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Growth Supplements</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>76.90000000000001</v>
-      </c>
-      <c r="E3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F3" t="n">
-        <v>88</v>
-      </c>
-      <c r="G3" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Linha Joie Fit</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Black Skull</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>124.9</v>
-      </c>
-      <c r="E4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F4" t="n">
-        <v>640</v>
-      </c>
-      <c r="G4" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="H4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="H4" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>sim</t>
         </is>
@@ -4604,112 +4604,112 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Linha Joie Fit</t>
+          <t>Amaze</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Max Titanium</t>
+          <t>Growth Supplements</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>89.90000000000001</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>310</v>
+        <v>88</v>
       </c>
       <c r="G5" t="n">
-        <v>4.4</v>
+        <v>4.6</v>
       </c>
       <c r="H5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>sim</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Linha Joie Fit</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>NÓS</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="D6" s="11" t="n">
-        <v>129.9</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="11" t="n">
-        <v>210</v>
-      </c>
-      <c r="G6" s="11" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H6" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="I6" s="11" t="inlineStr">
-        <is>
-          <t>nao</t>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Black Skull</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>124.9</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>640</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>sim</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Faciderm</t>
+          <t>Linha Joie Fit</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Black Skull</t>
+          <t>Max Titanium</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>74.90000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>210</v>
+        <v>310</v>
       </c>
       <c r="G7" t="n">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="H7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>nao</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Faciderm</t>
+          <t>Linha Joie Fit</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -4718,26 +4718,26 @@
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>149.9</v>
+        <v>129.9</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>95</v>
+        <v>210</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="H8" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>nao</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Redesenha o war room no estilo "capa técnica" (azul único, pipeline, selo)
Segue a referência visual enviada: navy quase-preto com grade blueprint, UM
azul de acento (#1187f0 — violeta/magenta removidos), bordas finas de 1px,
raio 10px, micro-labels em caixa alta com tracking largo e título bicolor.

Três elementos-assinatura novos, todos alimentados por dado real da rodada:
- render_pipeline(): COLETA » DIFF » ALERTA » AGENTE » AÇÃO, com a etapa
  acesa sendo a última que de fato aconteceu (linha de base acende DIFF;
  alerta aguardando autorização acende AÇÃO).
- render_seal(): selo circular com anel duplo, ticks radiais e a cadência
  configurada no centro.
- render_credbar(): rodapé com produtos/concorrentes monitorados (+ candidatos)
  e as fontes ativas na rodada, sinalizando "(simulado)" quando aplicável.

As cores categóricas dos gráficos (validadas p/ daltonismo) seguem intactas.
</commit_message>
<xml_diff>
--- a/war-room-concorrencia/contexto-e-apoio/arquivos-finais/war-room.xlsx
+++ b/war-room-concorrencia/contexto-e-apoio/arquivos-finais/war-room.xlsx
@@ -2411,7 +2411,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Gerado em 2026-08-01 10:11 UTC | cadência sugerida: 6h</t>
+          <t>Gerado em 2026-08-01 10:24 UTC | cadência sugerida: 6h</t>
         </is>
       </c>
     </row>
@@ -3027,7 +3027,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-01 10:11 UTC</t>
+          <t>2026-08-01 10:24 UTC</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-01 10:11 UTC</t>
+          <t>2026-08-01 10:24 UTC</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-01 10:11 UTC</t>
+          <t>2026-08-01 10:24 UTC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-01 10:11 UTC</t>
+          <t>2026-08-01 10:24 UTC</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-01 10:11 UTC</t>
+          <t>2026-08-01 10:24 UTC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-01 10:11 UTC</t>
+          <t>2026-08-01 10:24 UTC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3968,123 +3968,123 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Linha Joie Fit</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Black Skull</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>129.9</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>910</v>
+      </c>
+      <c r="G2" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Linha Joie Fit</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>NÓS</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" s="11" t="n">
+        <v>129.9</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>480</v>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H3" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>desconhecido</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Faciderm</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Black Skull</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
         <v>71.90000000000001</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E4" t="n">
         <v>20</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F4" t="n">
         <v>365</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G4" t="n">
         <v>4.6</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Faciderm</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Growth Supplements</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>68.90000000000001</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>12</v>
-      </c>
-      <c r="G3" t="n">
-        <v>4.4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>Faciderm</t>
-        </is>
-      </c>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>NÓS</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>149.9</v>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="11" t="n">
-        <v>210</v>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="H4" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="11" t="inlineStr">
-        <is>
-          <t>desconhecido</t>
-        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Amaze</t>
+          <t>Faciderm</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Black Skull</t>
+          <t>Growth Supplements</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>84.90000000000001</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>95</v>
+        <v>12</v>
       </c>
       <c r="G5" t="n">
-        <v>4.3</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Amaze</t>
+          <t>Faciderm</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
@@ -4093,19 +4093,19 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>99.90000000000001</v>
+        <v>149.9</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>340</v>
+        <v>210</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="H6" s="11" t="b">
         <v>1</v>
@@ -4119,7 +4119,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Linha Joie Fit</t>
+          <t>Amaze</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4131,22 +4131,22 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>129.9</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>910</v>
+        <v>95</v>
       </c>
       <c r="G7" t="n">
-        <v>4.8</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Linha Joie Fit</t>
+          <t>Amaze</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -4155,22 +4155,22 @@
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>129.9</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>480</v>
+        <v>340</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="H8" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
@@ -4499,7 +4499,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Faciderm</t>
+          <t>Linha Joie Fit</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4511,16 +4511,16 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>74.90000000000001</v>
+        <v>124.9</v>
       </c>
       <c r="E2" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>210</v>
+        <v>640</v>
       </c>
       <c r="G2" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
@@ -4532,44 +4532,44 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>Faciderm</t>
-        </is>
-      </c>
-      <c r="B3" s="11" t="inlineStr">
-        <is>
-          <t>NÓS</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" s="11" t="n">
-        <v>149.9</v>
-      </c>
-      <c r="E3" s="11" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Linha Joie Fit</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Max Titanium</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="11" t="n">
-        <v>95</v>
-      </c>
-      <c r="G3" s="11" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="H3" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="11" t="inlineStr">
-        <is>
-          <t>sim</t>
+      <c r="F3" t="n">
+        <v>310</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>nao</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Amaze</t>
+          <t>Linha Joie Fit</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
@@ -4578,166 +4578,166 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>99.90000000000001</v>
+        <v>129.9</v>
       </c>
       <c r="E4" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>150</v>
+        <v>210</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="H4" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>nao</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Faciderm</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Black Skull</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="E5" t="n">
+        <v>17</v>
+      </c>
+      <c r="F5" t="n">
+        <v>210</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Faciderm</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>NÓS</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>149.9</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H6" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
           <t>Amaze</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>NÓS</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>150</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H7" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Amaze</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Growth Supplements</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C8" t="n">
         <v>2</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D8" t="n">
         <v>76.90000000000001</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E8" t="n">
         <v>4</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F8" t="n">
         <v>88</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G8" t="n">
         <v>4.6</v>
       </c>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Linha Joie Fit</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Black Skull</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>124.9</v>
-      </c>
-      <c r="E6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F6" t="n">
-        <v>640</v>
-      </c>
-      <c r="G6" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="H6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Linha Joie Fit</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Max Titanium</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" t="n">
-        <v>89.90000000000001</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>310</v>
-      </c>
-      <c r="G7" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="H7" t="b">
-        <v>0</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>nao</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Linha Joie Fit</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>NÓS</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" s="11" t="n">
-        <v>129.9</v>
-      </c>
-      <c r="E8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="11" t="n">
-        <v>210</v>
-      </c>
-      <c r="G8" s="11" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H8" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="I8" s="11" t="inlineStr">
-        <is>
-          <t>nao</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona camada de efeitos neon/interativos ao war room (_fx_neon.py)
Ambiente: partículas em canvas com constelações e parallax de mouse, aurora
que deriva, scanline e spotlight que segue o cursor.
Lente: vidro (backdrop-filter) nos painéis e tilt 3D nos battlecards com
reflexo acompanhando o cursor.
Neon: border-beam girando na etapa ativa do pipeline, selo com anel girando e
sweep de radar, breathe pulsante nos itens críticos, pulso nas setas.
Movimento: revelação em cascata (IntersectionObserver), contadores animados
(só onde há número real), linha do gráfico se desenhando.
Popups: modal de detalhe do battlecard (payload dos mesmos alertas já
calculados), modal genérico de linha de tabela lendo os próprios th/td, e
tooltip nos pontos do gráfico.
Interativos: ripple, chips de filtro de severidade que filtram de verdade os
battlecards, e navegação das abas por teclado.

Tudo com fallback em prefers-reduced-motion mantendo as interações.
</commit_message>
<xml_diff>
--- a/war-room-concorrencia/contexto-e-apoio/arquivos-finais/war-room.xlsx
+++ b/war-room-concorrencia/contexto-e-apoio/arquivos-finais/war-room.xlsx
@@ -2411,7 +2411,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Gerado em 2026-08-01 10:24 UTC | cadência sugerida: 6h</t>
+          <t>Gerado em 2026-08-01 10:34 UTC | cadência sugerida: 6h</t>
         </is>
       </c>
     </row>
@@ -3027,7 +3027,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-01 10:24 UTC</t>
+          <t>2026-08-01 10:34 UTC</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-01 10:24 UTC</t>
+          <t>2026-08-01 10:34 UTC</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-01 10:24 UTC</t>
+          <t>2026-08-01 10:34 UTC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-01 10:24 UTC</t>
+          <t>2026-08-01 10:34 UTC</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-01 10:24 UTC</t>
+          <t>2026-08-01 10:34 UTC</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-01 10:24 UTC</t>
+          <t>2026-08-01 10:34 UTC</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3968,7 +3968,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Linha Joie Fit</t>
+          <t>Faciderm</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3980,111 +3980,111 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>129.9</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="E2" t="n">
+        <v>20</v>
+      </c>
+      <c r="F2" t="n">
+        <v>365</v>
+      </c>
+      <c r="G2" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Faciderm</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Growth Supplements</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="n">
-        <v>910</v>
-      </c>
-      <c r="G2" t="n">
-        <v>4.8</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>Linha Joie Fit</t>
-        </is>
-      </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="F3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Faciderm</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>NÓS</t>
         </is>
       </c>
-      <c r="C3" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="D3" s="11" t="n">
-        <v>129.9</v>
-      </c>
-      <c r="E3" s="11" t="n">
+      <c r="C4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>149.9</v>
+      </c>
+      <c r="E4" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="11" t="n">
-        <v>480</v>
-      </c>
-      <c r="G3" s="11" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H3" s="11" t="b">
-        <v>0</v>
-      </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="F4" s="11" t="n">
+        <v>210</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H4" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>desconhecido</t>
         </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Faciderm</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Black Skull</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>71.90000000000001</v>
-      </c>
-      <c r="E4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F4" t="n">
-        <v>365</v>
-      </c>
-      <c r="G4" t="n">
-        <v>4.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Faciderm</t>
+          <t>Amaze</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Growth Supplements</t>
+          <t>Black Skull</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>68.90000000000001</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>12</v>
+        <v>95</v>
       </c>
       <c r="G5" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Faciderm</t>
+          <t>Amaze</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
@@ -4093,19 +4093,19 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>149.9</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>210</v>
+        <v>340</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="H6" s="11" t="b">
         <v>1</v>
@@ -4119,7 +4119,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Amaze</t>
+          <t>Linha Joie Fit</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4131,22 +4131,22 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>84.90000000000001</v>
+        <v>129.9</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>95</v>
+        <v>910</v>
       </c>
       <c r="G7" t="n">
-        <v>4.3</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Amaze</t>
+          <t>Linha Joie Fit</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -4155,22 +4155,22 @@
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>99.90000000000001</v>
+        <v>129.9</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>340</v>
+        <v>480</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="H8" s="11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
@@ -4499,7 +4499,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Linha Joie Fit</t>
+          <t>Faciderm</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4511,65 +4511,65 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>124.9</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="E2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F2" t="n">
+        <v>210</v>
+      </c>
+      <c r="G2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Faciderm</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>NÓS</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F2" t="n">
-        <v>640</v>
-      </c>
-      <c r="G2" t="n">
+      <c r="D3" s="11" t="n">
+        <v>149.9</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>95</v>
+      </c>
+      <c r="G3" s="11" t="n">
         <v>4.7</v>
       </c>
-      <c r="H2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="H3" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Linha Joie Fit</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Max Titanium</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>89.90000000000001</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>310</v>
-      </c>
-      <c r="G3" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="H3" t="b">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>nao</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Linha Joie Fit</t>
+          <t>Amaze</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
@@ -4578,166 +4578,166 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>129.9</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="E4" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>210</v>
+        <v>150</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="H4" s="11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>sim</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Faciderm</t>
+          <t>Amaze</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Growth Supplements</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="n">
+        <v>88</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Linha Joie Fit</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>Black Skull</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="n">
-        <v>74.90000000000001</v>
-      </c>
-      <c r="E5" t="n">
-        <v>17</v>
-      </c>
-      <c r="F5" t="n">
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>124.9</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>640</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Linha Joie Fit</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Max Titanium</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>310</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nao</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Linha Joie Fit</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>NÓS</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>129.9</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="11" t="n">
         <v>210</v>
       </c>
-      <c r="G5" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>Faciderm</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>NÓS</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" s="11" t="n">
-        <v>149.9</v>
-      </c>
-      <c r="E6" s="11" t="n">
+      <c r="G8" s="11" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H8" s="11" t="b">
         <v>0</v>
       </c>
-      <c r="F6" s="11" t="n">
-        <v>95</v>
-      </c>
-      <c r="G6" s="11" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="H6" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" s="11" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Amaze</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>NÓS</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="11" t="n">
-        <v>99.90000000000001</v>
-      </c>
-      <c r="E7" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="11" t="n">
-        <v>150</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="H7" s="11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Amaze</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Growth Supplements</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" t="n">
-        <v>76.90000000000001</v>
-      </c>
-      <c r="E8" t="n">
-        <v>4</v>
-      </c>
-      <c r="F8" t="n">
-        <v>88</v>
-      </c>
-      <c r="G8" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H8" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>sim</t>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>nao</t>
         </is>
       </c>
     </row>

</xml_diff>